<commit_message>
Agregar correcciones en Anexo B
</commit_message>
<xml_diff>
--- a/02_Inspeccion/AnexoB_registro_defectos.xlsx
+++ b/02_Inspeccion/AnexoB_registro_defectos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ISR401-PFC-ERS-EquipoD\02_Inspeccion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F41BBB8E-7D26-4804-9076-7AC7CEC5EC83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0023685-5AFB-4432-81BE-68B54568EE65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{586D01C1-B356-4565-9C45-D63985A7303B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C48A4765-B3C5-407D-9115-3CEDE7100ED7}"/>
   </bookViews>
   <sheets>
     <sheet name="AnexoB_registro_defectos" sheetId="1" r:id="rId1"/>
@@ -20,18 +20,21 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="49">
   <si>
     <t>Anexo B - Registro consolidado de defectos de la inspeccion Fagan;;;;;;;</t>
   </si>
   <si>
+    <t>Documento inspeccionado;ERS_v1.0.pdf (identico a ERS_SRS_2A_v1.0.pdf);Paginas efectivas;147;Fecha de la reunion;2026-08-09;Moderador;Morales Sanchez Gary Alejandro</t>
+  </si>
+  <si>
     <t>Minimo exigido por la guia;15 defectos unicos con al menos 3 criticos o mayores;Consolidado obtenido;18 defectos unicos;Criticos;2;Mayores;12</t>
   </si>
   <si>
-    <t>Nota;La columna Correccion se completa en la fase de correccion posterior. La inspeccion detecta</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> no corrige.;;;;;;</t>
+    <t>Nota;La columna Correccion se completo en la fase de correccion posterior (Seccion 5 y RFC-01/02/03). La inspeccion detecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> no corrigio.;;;;;;</t>
   </si>
   <si>
     <t>;;;;;;;</t>
@@ -40,58 +43,121 @@
     <t>N.o;Seccion del ERS;Descripcion del defecto;Tipo;Severidad;Requisito afectado;Detectado por;Correccion</t>
   </si>
   <si>
-    <t>D-01;1.2 Alcance del producto (linea 392);El MVP se define como cobertura de "al menos el 60 % de los RF de prioridad Debe tener" sin enumerar cuales de los 15 RF Must lo integran. El alcance admite multiples subconjuntos validos. Ademas usa "Debe tener" donde el resto del documento usa "Must".;Ambiguedad;Menor;Alcance del MVP;Morales;</t>
-  </si>
-  <si>
-    <t>D-02;1.2 Alcance del producto (lineas 388 y 390);"Sugerencias inteligentes para completar perfiles" y "Recomendaciones basicas de cuidado" figuran como alcance incluido pero ningun RF del catalogo RF-01 a RF-25 las especifica.;Completitud;Mayor;RF-01 a RF-25 (ausentes);Morales;</t>
-  </si>
-  <si>
-    <t>D-03;1.2 Alcance vs 3.2 RF-07 (lineas 374 y 1344);El alcance declara comunicacion entre propietarios adoptantes interesados en cruza refugios y veterinarias. RF-07 lista como actores solo Propietario Adoptante e Interesado en cruza. Refugio y Veterinaria quedan fuera del requisito.;Consistencia;Mayor;RF-07;Morales;</t>
-  </si>
-  <si>
-    <t>D-04;2.6 Suposiciones y dependencias (linea 830);La suposicion "el volumen inicial de usuarios permitira operar con una infraestructura basica de hosting" no define volumen ni que significa basica. No puede comprobarse y tensiona con RNF-12 que exige 300 usuarios concurrentes.;Verificabilidad;Menor;RNF-12;Morales;</t>
-  </si>
-  <si>
-    <t>D-05;2.4.2 Conflictos entre stakeholders (linea 791);La estrategia de gestion declara "mecanismos basicos para reportar interacciones inadecuadas" pero no existe ningun RF de reporte o denuncia de usuarios. Estrategia sin requisito destino.;Trazabilidad;Mayor;RF ausente (reporte de usuarios);Morales;</t>
-  </si>
-  <si>
-    <t>D-06;2.6 Dependencias vs 3.3 RNF-09 y 3.5 RD-08 (lineas 837 y 1778);La dependencia externa se enuncia en condicional ("podria requerirse la integracion con un servicio externo de notificaciones") mientras RNF-09 compromete en firme WhatsApp Business API y RD-08 lo eleva a restriccion de diseno. Es un servicio de pago sin suposicion de costo ni presupuesto que lo sostenga.;Factibilidad;Mayor;RNF-09 y RD-08;Morales;</t>
-  </si>
-  <si>
-    <t>D-07;3.2 RF-23 (linea 1599);La alerta se dispara ante "una disparidad de tamano significativa" sin umbral cuantificado. El criterio de verificacion repite el mismo termino y propaga la ambiguedad a la prueba. Requisito Must ligado a seguridad fisica del animal.;Ambiguedad;Mayor;RF-23;Sanchez;</t>
-  </si>
-  <si>
-    <t>D-08;3.2 RF-01 vs RF-04 y RF-06 (lineas 1250 1295 1327);RF-04 filtra por temperamento y RF-06 evalua comportamiento pero RF-01 no incluye ninguno de los dos entre las entradas del registro. Se consume un dato que ningun RF captura.;Completitud;Mayor;RF-01 RF-04 RF-06;Sanchez;</t>
-  </si>
-  <si>
-    <t>D-09;3.2 RF-25 vs 3.3 RNF-16 (lineas 1631 1635);RF-25 publica un aviso visible publicamente que incluye datos de contacto. RNF-16 exige el 100 % de los perfiles con ubicacion y contacto ocultos por defecto y tiene prioridad Must frente al Could de RF-25. Ademas RF-25 no consta en la tabla legal RL-05 sobre minimizacion (LOPDP Art. 10 lit. e).;Consistencia;Critico;RF-25 y RNF-16;Sanchez;</t>
-  </si>
-  <si>
-    <t>D-10;3.2 RF-01 (linea 1255);El criterio de verificacion "registrar una mascota con datos validos" no define campos obligatorios ni reglas de validez por lo que la prueba no es decidible. El propio ERS reconoce el hueco en la estrategia del conflicto de la linea 779.;Verificabilidad;Menor;RF-01;Sanchez;</t>
-  </si>
-  <si>
-    <t>D-11;3.2 RF-06 (linea 1329);El origen se declara como rango "EV-01 a EV-08" donde los otros 24 RF enumeran evidencia por evidencia. Impide comprobar que cada EV sustenta el requisito y no coincide con la fila TR-06 de la matriz que solo cita EV-04 EV-05 EV-06 y EV-08.;Trazabilidad;Mayor;RF-06;Sanchez;</t>
-  </si>
-  <si>
-    <t>D-12;3.2 CU-08 y RF-07 (lineas 2853 1213 1350);El alcance y CU-08 comprometen un clasificador de lenguaje ofensivo en espanol. No hay RNF de exactitud para moderacion (RNF-06 cubre cruza y RNF-07 imagenes) ni suposicion sobre datos de entrenamiento y todo depende de RF-07 cuya prioridad es Could.;Factibilidad;Mayor;RF-07 y CU-08;Sanchez;</t>
-  </si>
-  <si>
-    <t>D-13;3.3 RNF-12 (linea 1817);La descripcion normativa usa "sin degradar significativamente el tiempo de respuesta definido en RNF-03". El valor objetivo si esta cuantificado pero la clausula que se contrata contiene un termino de grado indefinido.;Ambiguedad;Menor;RNF-12;Cedeno;</t>
-  </si>
-  <si>
-    <t>D-14;3.3 RNF-15 (linea 1856);RNF-15 exige explicabilidad cuando un mensaje es marcado por el componente de moderacion automatica pero ningun RF especifica esa moderacion. La funcion solo existe en la tabla de interfaces de software y en CU-08. RNF sin requisito funcional padre.;Completitud;Mayor;RNF-15;Cedeno;</t>
-  </si>
-  <si>
-    <t>D-15;Apendice B.3 fila EV-04 (lineas 6265 y 6281);La fila EV-04 declara al participante como VET-02 y en la misma fila nombra el archivo 2026-05-17_Veterinario_VET-04_TranscripcionEntrevista.txt. Contradiccion interna en una sola fila. Agravante: el documento se entrega con una nota de consistencia pendiente de verificacion sin resolver.;Consistencia;Critico;EV-04 y trazabilidad de evidencias;Cedeno;</t>
-  </si>
-  <si>
-    <t>D-16;3.3 RNF-02 (linea 1691);El criterio de verificacion exige monitorear la disponibilidad durante un mes de operacion. El sistema no esta en produccion y el PFC no contempla un mes de operacion real ni se declara entorno o suposicion que lo permita. Requisito inverificable en la practica.;Verificabilidad;Mayor;RNF-02;Cedeno;</t>
-  </si>
-  <si>
-    <t>D-17;Apendice B.3 y Apendice D (lineas 6281 4159 6546);La referencia cruzada a la tabla de evidencias no resuelve y el PDF imprime "??" en la pagina 126 (confirmado en el log de compilacion). Ademas se afirma que la matriz debe coincidir con 04_Trazabilidad/matriz_trazabilidad.csv y se citan priorizacion_moscow_kano.csv codificacion_tematica.csv y fichas_tecnicas.csv: ninguno de los cuatro esta en el repositorio ni se da URL.;Trazabilidad;Mayor;Apendice D y matriz de trazabilidad;Cedeno;</t>
-  </si>
-  <si>
-    <t>D-18;3.3 Tabla de cobertura ISO/IEC 25010:2023 (linea 1648);La tabla dice cubrir las nueve caracteristicas de ISO/IEC 25010:2023 pero lista Portabilidad como caracteristica de primer nivel (en la revision 2023 es subcaracteristica de Flexibilidad) y omite Inocuidad (Safety). El mapeo de calidad se construyo sobre la estructura de la version 2011.;Factibilidad;Mayor;Tabla de cobertura 25010 y RNF-11;Cedeno;</t>
+    <t>D-01;1.2 Alcance del producto (linea 392);El MVP se define como cobertura de "al menos el 60 % de los RF de prioridad Debe tener" sin enumerar cuales de los 15 RF Must lo integran. El alcance admite multiples subconjuntos validos. Ademas usa "Debe tener" donde el resto del documento usa "Must".;Ambiguedad;Menor;Alcance del MVP;Morales;No corregido en esta iteracion. Justificacion: la seleccion exacta del 60 % de RF Must se resuelve en el ejercicio de priorizacion (Kano/WSJF) del Apendice, posterior a esta validacion, no en el ERS.</t>
+  </si>
+  <si>
+    <t>D-02;1.2 Alcance del producto (lineas 388 y 390);"Sugerencias inteligentes para completar perfiles" y "Recomendaciones basicas de cuidado" figuran como alcance incluido pero ningun RF del catalogo RF-01 a RF-25 las especifica.;Completitud;Mayor;RF-01 a RF-25 (ausentes);Morales;Tramitado via RFC-01 (CCB). Se retiran del alcance incluido "Sugerencias inteligentes para completar perfiles" y "Recomendaciones basicas de cuidado": ninguna cuenta con evidencia de campo que la respalde ni figura en la matriz de trazabilidad; el CCB decidio no ampliar el alcance sin elicitacion previa.</t>
+  </si>
+  <si>
+    <t>D-03;1.2 Alcance vs 3.2 RF-07 (lineas 374 y 1344);El alcance declara comunicacion entre propietarios adoptantes interesados en cruza refugios y veterinarias. RF-07 lista como actores solo Propietario Adoptante e Interesado en cruza. Refugio y Veterinaria quedan fuera del requisito.;Consistencia;Mayor;RF-07;Morales;Correccion directa. Actor de RF-07 ampliado de ""Propietario de mascota</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Adoptante</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Interesado en cruza"" a ""Propietario de mascota</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Interesado en cruza</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Refugio</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Veterinaria"".</t>
+  </si>
+  <si>
+    <t>D-04;2.6 Suposiciones y dependencias (linea 830);La suposicion "el volumen inicial de usuarios permitira operar con una infraestructura basica de hosting" no define volumen ni que significa basica. No puede comprobarse y tensiona con RNF-12 que exige 300 usuarios concurrentes.;Verificabilidad;Menor;RNF-12;Morales;No corregido en esta iteracion. Justificacion: el dimensionamiento de infraestructura es una decision de diseno arquitectonico, fuera del nivel de abstraccion de un ERS; se difiere al documento de arquitectura.</t>
+  </si>
+  <si>
+    <t>D-05;2.4.2 Conflictos entre stakeholders (linea 791);La estrategia de gestion declara "mecanismos basicos para reportar interacciones inadecuadas" pero no existe ningun RF de reporte o denuncia de usuarios. Estrategia sin requisito destino.;Trazabilidad;Mayor;RF ausente (reporte de usuarios);Morales;Correccion directa. Estrategia de conflicto reformulada: se retira la promesa de un mecanismo de reporte inexistente y se ancla a la conservacion del historial de conversacion como respaldo del usuario ante disputas (RF-07).</t>
+  </si>
+  <si>
+    <t>D-06;2.6 Dependencias vs 3.3 RNF-09 y 3.5 RD-08 (lineas 837 y 1778);La dependencia externa se enuncia en condicional ("podria requerirse la integracion con un servicio externo de notificaciones") mientras RNF-09 compromete en firme WhatsApp Business API y RD-08 lo eleva a restriccion de diseno. Es un servicio de pago sin suposicion de costo ni presupuesto que lo sostenga.;Factibilidad;Mayor;RNF-09 y RD-08;Morales;Tramitado via RFC-02 (CCB). RNF-09 y RD-08 reformulados sin mencion nominal a WhatsApp Business API; se retira el compromiso con un proveedor unico de pago y se eleva el canal de respaldo in-app de recomendacion a obligacion.</t>
+  </si>
+  <si>
+    <t>D-07;3.2 RF-23 (linea 1599);La alerta se dispara ante "una disparidad de tamano significativa" sin umbral cuantificado. El criterio de verificacion repite el mismo termino y propaga la ambiguedad a la prueba. Requisito Must ligado a seguridad fisica del animal.;Ambiguedad;Mayor;RF-23;Sanchez;Correccion directa. Umbral cuantificado en RF-23: "diferencia de peso corporal estimado igual o superior al 40 % entre ambas mascotas, o presencia de enfermedad contagiosa activa"; mismo umbral aplicado al criterio de verificacion.</t>
+  </si>
+  <si>
+    <t>D-08;3.2 RF-01 vs RF-04 y RF-06 (lineas 1250 1295 1327);RF-04 filtra por temperamento y RF-06 evalua comportamiento pero RF-01 no incluye ninguno de los dos entre las entradas del registro. Se consume un dato que ningun RF captura.;Completitud;Mayor;RF-01 RF-04 RF-06;Sanchez;Correccion directa. Entradas de RF-01 ampliadas de ""Nombre</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> especie</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> raza</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> sexo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> edad</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> estado reproductivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> fotografias</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> descripcion"" a ""Nombre</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> temperamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> comportamiento observado</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> descripcion"".</t>
+  </si>
+  <si>
+    <t>D-09;3.2 RF-25 vs 3.3 RNF-16 (lineas 1631 1635);RF-25 publica un aviso visible publicamente que incluye datos de contacto. RNF-16 exige el 100 % de los perfiles con ubicacion y contacto ocultos por defecto y tiene prioridad Must frente al Could de RF-25. Ademas RF-25 no consta en la tabla legal RL-05 sobre minimizacion (LOPDP Art. 10 lit. e).;Consistencia;Critico;RF-25 y RNF-16;Sanchez;Tramitado via RFC-03 (CCB). El CCB resolvio el conflicto a favor de RNF-16 por jerarquia de prioridad y fundamento legal: RF-25 ya no publica contacto directo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> el contacto se canaliza via mensajeria interna (RF-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> elevado de Could a Must); se crea CU-14.</t>
+  </si>
+  <si>
+    <t>D-10;3.2 RF-01 (linea 1255);El criterio de verificacion "registrar una mascota con datos validos" no define campos obligatorios ni reglas de validez por lo que la prueba no es decidible. El propio ERS reconoce el hueco en la estrategia del conflicto de la linea 779.;Verificabilidad;Menor;RF-01;Sanchez;No corregido en esta iteracion. Justificacion: la validacion campo por campo de RF-01 corresponde al diccionario de datos del diseno detallado; el ERS especifica el requisito, no las reglas de validacion de cada campo.</t>
+  </si>
+  <si>
+    <t>D-11;3.2 RF-06 (linea 1329);El origen se declara como rango "EV-01 a EV-08" donde los otros 24 RF enumeran evidencia por evidencia. Impide comprobar que cada EV sustenta el requisito y no coincide con la fila TR-06 de la matriz que solo cita EV-04 EV-05 EV-06 y EV-08.;Trazabilidad;Mayor;RF-06;Sanchez;Correccion directa. Origen de RF-06 corregido de "EV-01 a EV-08, EV-11, EV-13, EV-14, EV-15, EV-16" a enumeracion explicita "EV-04, EV-05, EV-06, EV-08", coherente con la fila TR-06 de la matriz de trazabilidad.</t>
+  </si>
+  <si>
+    <t>D-12;3.2 CU-08 y RF-07 (lineas 2853 1213 1350);El alcance y CU-08 comprometen un clasificador de lenguaje ofensivo en espanol. No hay RNF de exactitud para moderacion (RNF-06 cubre cruza y RNF-07 imagenes) ni suposicion sobre datos de entrenamiento y todo depende de RF-07 cuya prioridad es Could.;Factibilidad;Mayor;RF-07 y CU-08;Sanchez;Correccion directa (ligada a RFC-01). Se anade en Suposiciones (Seccion 2.6): ""Se asume la disponibilidad de un conjunto de mensajes reales o sinteticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> previamente etiquetados</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> suficiente para entrenar y evaluar el componente de moderacion automatica de texto en espanol""; RF-07 se eleva a Must y la moderacion queda especificada en el nuevo RF-26.</t>
+  </si>
+  <si>
+    <t>D-13;3.3 RNF-12 (linea 1817);La descripcion normativa usa "sin degradar significativamente el tiempo de respuesta definido en RNF-03". El valor objetivo si esta cuantificado pero la clausula que se contrata contiene un termino de grado indefinido.;Ambiguedad;Menor;RNF-12;Cedeno;No corregido en esta iteracion. Justificacion: el valor objetivo de RNF-12 ya esta cuantificado (&lt;=3 s P95 con 300 usuarios concurrentes); ese valor gobierna la verificacion con independencia del adjetivo impreciso en la descripcion narrativa.</t>
+  </si>
+  <si>
+    <t>D-14;3.3 RNF-15 (linea 1856);RNF-15 exige explicabilidad cuando un mensaje es marcado por el componente de moderacion automatica pero ningun RF especifica esa moderacion. La funcion solo existe en la tabla de interfaces de software y en CU-08. RNF sin requisito funcional padre.;Completitud;Mayor;RNF-15;Cedeno;Tramitado via RFC-01 (CCB). Se crea el nuevo RF-26 (moderar automaticamente los mensajes entre usuarios) y RNF-15 queda vinculado a el como requisito funcional padre.</t>
+  </si>
+  <si>
+    <t>D-15;Apendice B.3 fila EV-04 (lineas 6265 y 6281);La fila EV-04 declara al participante como VET-02 y en la misma fila nombra el archivo 2026-05-17_Veterinario_VET-04_TranscripcionEntrevista.txt. Contradiccion interna en una sola fila. Agravante: el documento se entrega con una nota de consistencia pendiente de verificacion sin resolver.;Consistencia;Critico;EV-04 y trazabilidad de evidencias;Cedeno;Correccion directa. Nombre de archivo corregido de ""...Veterinario_VET-04_TranscripcionEntrevista.txt"" a ""...Veterinario_VET-02_TranscripcionEntrevista.txt""</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> coherente con el participante VET-02 de la fila; se retira la nota de consistencia pendiente.</t>
+  </si>
+  <si>
+    <t>D-16;3.3 RNF-02 (linea 1691);El criterio de verificacion exige monitorear la disponibilidad durante un mes de operacion. El sistema no esta en produccion y el PFC no contempla un mes de operacion real ni se declara entorno o suposicion que lo permita. Requisito inverificable en la practica.;Verificabilidad;Mayor;RNF-02;Cedeno;Correccion directa. Criterio de verificacion reformulado de ""monitorear la disponibilidad del sistema durante un mes de operacion"" a ""monitorear la disponibilidad del entorno de pruebas o staging durante un periodo minimo de 7 dias continuos</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> complementado con pruebas de resiliencia que proyecten la disponibilidad esperada en produccion"".</t>
+  </si>
+  <si>
+    <t>D-17;Apendice B.3 y Apendice D (lineas 6281 4159 6546);La referencia cruzada a la tabla de evidencias no resuelve y el PDF imprime "??" en la pagina 126 (confirmado en el log de compilacion). Ademas se afirma que la matriz debe coincidir con 04_Trazabilidad/matriz_trazabilidad.csv y se citan priorizacion_moscow_kano.csv codificacion_tematica.csv y fichas_tecnicas.csv: ninguno de los cuatro esta en el repositorio ni se da URL.;Trazabilidad;Mayor;Apendice D y matriz de trazabilidad;Cedeno;Correccion directa. Se agrega \label{tab:evidencias} a la tabla del Apendice B.3 (resuelve la referencia rota, pagina 126); se suben matriz_trazabilidad.csv, priorizacion_moscow_kano.csv, codificacion_tematica.csv y fichas_tecnicas.csv a 04_Trazabilidad/.</t>
+  </si>
+  <si>
+    <t>D-18;3.3 Tabla de cobertura ISO/IEC 25010:2023 (linea 1648);La tabla dice cubrir las nueve caracteristicas de ISO/IEC 25010:2023 pero lista Portabilidad como caracteristica de primer nivel (en la revision 2023 es subcaracteristica de Flexibilidad) y omite Inocuidad (Safety). El mapeo de calidad se construyo sobre la estructura de la version 2011.;Factibilidad;Mayor;Tabla de cobertura 25010 y RNF-11;Cedeno;Correccion directa. Portabilidad reclasificada como subcaracteristica de Flexibilidad; se incorpora Inocuidad (Safety) como caracteristica independiente (sin RNF asociado en esta version); verificado por Cedeno contra el texto oficial de la norma antes de cerrar la v1.1.</t>
   </si>
   <si>
     <t>Resumen por severidad;Critico;2;Mayor;12;Menor;4;Total 18</t>
@@ -101,9 +167,6 @@
   </si>
   <si>
     <t>Resumen por inspector;Morales;6;Sanchez;6;Cedeno;6;Total 18</t>
-  </si>
-  <si>
-    <t>Documento inspeccionado;ERS_SRS_2A_v1.0.pdf;Paginas efectivas;147;Fecha de la reunion;2026-08-09;Moderador;Morales Sanchez Gary Alejandro</t>
   </si>
 </sst>
 </file>
@@ -943,151 +1006,235 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{532A18A6-A4EA-4652-AFE6-11D5F37E5DFE}">
-  <dimension ref="A1:B28"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{597E68FB-A1AD-4108-9496-152688DFF40C}">
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" t="s">
+        <v>22</v>
+      </c>
+      <c r="E14" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" t="s">
+        <v>24</v>
+      </c>
+      <c r="G14" t="s">
+        <v>25</v>
+      </c>
+      <c r="H14" t="s">
+        <v>26</v>
+      </c>
+      <c r="I14" t="s">
+        <v>20</v>
+      </c>
+      <c r="J14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K14" t="s">
+        <v>22</v>
+      </c>
+      <c r="L14" t="s">
+        <v>23</v>
+      </c>
+      <c r="M14" t="s">
+        <v>24</v>
+      </c>
+      <c r="N14" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="O14" t="s">
+        <v>28</v>
+      </c>
+      <c r="P14" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>